<commit_message>
Bug solved, physiological results in sse28multidoftplus. Testing logSSE
</commit_message>
<xml_diff>
--- a/data/UMG_NSTEMI_Dataset.xlsx
+++ b/data/UMG_NSTEMI_Dataset.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="IDs"/>
@@ -331,13 +331,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -413,13 +419,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -432,9 +438,6 @@
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -487,14 +490,14 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="20" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf xfId="0" numFmtId="20" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="20" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="20" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -801,7 +804,7 @@
   <dimension ref="A1:A99"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -840,7 +843,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="9" t="s">
         <v>10</v>
       </c>
     </row>
@@ -870,7 +873,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="12" t="s">
         <v>16</v>
       </c>
     </row>
@@ -880,7 +883,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="15" t="s">
         <v>18</v>
       </c>
     </row>
@@ -900,7 +903,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="20" t="s">
+      <c r="A20" s="19" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1312,21 +1315,21 @@
   <dimension ref="A1:O99"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -1436,10 +1439,10 @@
       <c r="C4" s="1">
         <v>130.08</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
@@ -1557,9 +1560,9 @@
       <c r="D8" s="1">
         <v>81.75</v>
       </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -1650,9 +1653,9 @@
       <c r="D11" s="1">
         <v>129.92</v>
       </c>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -1672,10 +1675,10 @@
       <c r="C12" s="1">
         <v>153.53</v>
       </c>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
@@ -1804,8 +1807,8 @@
       <c r="E16" s="1">
         <v>178.28</v>
       </c>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -1859,9 +1862,9 @@
       <c r="D18" s="1">
         <v>155.58</v>
       </c>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -1890,7 +1893,7 @@
       <c r="F19" s="1">
         <v>128.43</v>
       </c>
-      <c r="G19" s="7"/>
+      <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -1904,7 +1907,7 @@
       <c r="A20" s="1">
         <v>18.5</v>
       </c>
-      <c r="B20" s="21">
+      <c r="B20" s="20">
         <v>33</v>
       </c>
       <c r="C20" s="1">
@@ -1916,8 +1919,8 @@
       <c r="E20" s="1">
         <v>106.27</v>
       </c>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
@@ -1943,8 +1946,8 @@
       <c r="E21" s="1">
         <v>106.47</v>
       </c>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -2000,9 +2003,9 @@
       <c r="D23" s="1">
         <v>154.18</v>
       </c>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
@@ -2028,8 +2031,8 @@
       <c r="E24" s="1">
         <v>106.42</v>
       </c>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
@@ -2058,7 +2061,7 @@
       <c r="F25" s="1">
         <v>106.42</v>
       </c>
-      <c r="G25" s="7"/>
+      <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
@@ -2276,8 +2279,8 @@
       <c r="E32" s="1">
         <v>73.05</v>
       </c>
-      <c r="F32" s="7"/>
-      <c r="G32" s="7"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
@@ -2303,8 +2306,8 @@
       <c r="E33" s="1">
         <v>106.9</v>
       </c>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
@@ -2327,9 +2330,9 @@
       <c r="D34" s="1">
         <v>57.35</v>
       </c>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="7"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
@@ -2355,8 +2358,8 @@
       <c r="E35" s="1">
         <v>105.33</v>
       </c>
-      <c r="F35" s="7"/>
-      <c r="G35" s="7"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
@@ -2385,7 +2388,7 @@
       <c r="F36" s="1">
         <v>67.93333333334886</v>
       </c>
-      <c r="G36" s="7"/>
+      <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
@@ -2408,9 +2411,9 @@
       <c r="D37" s="1">
         <v>92.18333333329065</v>
       </c>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
@@ -2436,8 +2439,8 @@
       <c r="E38" s="1">
         <v>165.81666666670935</v>
       </c>
-      <c r="F38" s="7"/>
-      <c r="G38" s="7"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
@@ -2466,7 +2469,7 @@
       <c r="F39" s="1">
         <v>94.74999999994179</v>
       </c>
-      <c r="G39" s="7"/>
+      <c r="G39" s="2"/>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
@@ -2563,7 +2566,7 @@
       <c r="F42" s="1">
         <v>71.08333333331393</v>
       </c>
-      <c r="G42" s="7"/>
+      <c r="G42" s="2"/>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
@@ -2592,7 +2595,7 @@
       <c r="F43" s="1">
         <v>93.51666666660458</v>
       </c>
-      <c r="G43" s="7"/>
+      <c r="G43" s="2"/>
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
@@ -2618,8 +2621,8 @@
       <c r="E44" s="1">
         <v>70.04999999993015</v>
       </c>
-      <c r="F44" s="7"/>
-      <c r="G44" s="7"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
@@ -2932,7 +2935,7 @@
       <c r="F53" s="1">
         <v>151.9000000000815</v>
       </c>
-      <c r="G53" s="7"/>
+      <c r="G53" s="2"/>
       <c r="H53" s="2"/>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
@@ -3064,7 +3067,7 @@
       <c r="F57" s="1">
         <v>115.15000000008149</v>
       </c>
-      <c r="G57" s="7"/>
+      <c r="G57" s="2"/>
       <c r="H57" s="2"/>
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
@@ -3157,7 +3160,7 @@
       <c r="F60" s="1">
         <v>85.483333333279</v>
       </c>
-      <c r="G60" s="7"/>
+      <c r="G60" s="2"/>
       <c r="H60" s="2"/>
       <c r="I60" s="2"/>
       <c r="J60" s="2"/>
@@ -3186,7 +3189,7 @@
       <c r="F61" s="1">
         <v>78.96666666667443</v>
       </c>
-      <c r="G61" s="7"/>
+      <c r="G61" s="2"/>
       <c r="H61" s="2"/>
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
@@ -3215,7 +3218,7 @@
       <c r="F62" s="1">
         <v>72.63333333330229</v>
       </c>
-      <c r="G62" s="7"/>
+      <c r="G62" s="2"/>
       <c r="H62" s="2"/>
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
@@ -3244,7 +3247,7 @@
       <c r="F63" s="1">
         <v>73.78333333320916</v>
       </c>
-      <c r="G63" s="7"/>
+      <c r="G63" s="2"/>
       <c r="H63" s="2"/>
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
@@ -3494,8 +3497,8 @@
       <c r="E70" s="1">
         <v>45.766666666720994</v>
       </c>
-      <c r="F70" s="7"/>
-      <c r="G70" s="7"/>
+      <c r="F70" s="2"/>
+      <c r="G70" s="2"/>
       <c r="H70" s="2"/>
       <c r="I70" s="2"/>
       <c r="J70" s="2"/>
@@ -3521,8 +3524,8 @@
       <c r="E71" s="1">
         <v>56.850000000034925</v>
       </c>
-      <c r="F71" s="7"/>
-      <c r="G71" s="7"/>
+      <c r="F71" s="2"/>
+      <c r="G71" s="2"/>
       <c r="H71" s="2"/>
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
@@ -3579,8 +3582,8 @@
       <c r="E73" s="1">
         <v>41.43333333340706</v>
       </c>
-      <c r="F73" s="7"/>
-      <c r="G73" s="7"/>
+      <c r="F73" s="2"/>
+      <c r="G73" s="2"/>
       <c r="H73" s="2"/>
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
@@ -3648,7 +3651,7 @@
       <c r="F75" s="1">
         <v>71.33333333343035</v>
       </c>
-      <c r="G75" s="21">
+      <c r="G75" s="20">
         <v>84</v>
       </c>
       <c r="H75" s="1">
@@ -3687,7 +3690,7 @@
       <c r="F76" s="1">
         <v>82.66666666668607</v>
       </c>
-      <c r="G76" s="7"/>
+      <c r="G76" s="2"/>
       <c r="H76" s="2"/>
       <c r="I76" s="2"/>
       <c r="J76" s="2"/>
@@ -3710,9 +3713,9 @@
       <c r="D77" s="1">
         <v>36.18333333340706</v>
       </c>
-      <c r="E77" s="7"/>
-      <c r="F77" s="7"/>
-      <c r="G77" s="7"/>
+      <c r="E77" s="2"/>
+      <c r="F77" s="2"/>
+      <c r="G77" s="2"/>
       <c r="H77" s="2"/>
       <c r="I77" s="2"/>
       <c r="J77" s="2"/>
@@ -3771,8 +3774,8 @@
       <c r="E79" s="1">
         <v>61.28333333332557</v>
       </c>
-      <c r="F79" s="7"/>
-      <c r="G79" s="7"/>
+      <c r="F79" s="2"/>
+      <c r="G79" s="2"/>
       <c r="H79" s="2"/>
       <c r="I79" s="2"/>
       <c r="J79" s="2"/>
@@ -4043,8 +4046,8 @@
       <c r="E87" s="1">
         <v>60.93333333340706</v>
       </c>
-      <c r="F87" s="7"/>
-      <c r="G87" s="7"/>
+      <c r="F87" s="2"/>
+      <c r="G87" s="2"/>
       <c r="H87" s="2"/>
       <c r="I87" s="2"/>
       <c r="J87" s="2"/>
@@ -4200,8 +4203,8 @@
       <c r="E92" s="1">
         <v>58.750000000116415</v>
       </c>
-      <c r="F92" s="7"/>
-      <c r="G92" s="7"/>
+      <c r="F92" s="2"/>
+      <c r="G92" s="2"/>
       <c r="H92" s="2"/>
       <c r="I92" s="2"/>
       <c r="J92" s="2"/>
@@ -4227,8 +4230,8 @@
       <c r="E93" s="1">
         <v>53.60000000009313</v>
       </c>
-      <c r="F93" s="7"/>
-      <c r="G93" s="7"/>
+      <c r="F93" s="2"/>
+      <c r="G93" s="2"/>
       <c r="H93" s="2"/>
       <c r="I93" s="2"/>
       <c r="J93" s="2"/>
@@ -4285,8 +4288,8 @@
       <c r="E95" s="1">
         <v>56.08333333331393</v>
       </c>
-      <c r="F95" s="7"/>
-      <c r="G95" s="7"/>
+      <c r="F95" s="2"/>
+      <c r="G95" s="2"/>
       <c r="H95" s="2"/>
       <c r="I95" s="2"/>
       <c r="J95" s="2"/>
@@ -4345,8 +4348,8 @@
       <c r="E97" s="1">
         <v>61.96666666661622</v>
       </c>
-      <c r="F97" s="7"/>
-      <c r="G97" s="7"/>
+      <c r="F97" s="2"/>
+      <c r="G97" s="2"/>
       <c r="H97" s="2"/>
       <c r="I97" s="2"/>
       <c r="J97" s="2"/>
@@ -4441,21 +4444,21 @@
   <dimension ref="A1:O99"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -4565,10 +4568,10 @@
       <c r="C4" s="1">
         <v>0.158</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
@@ -4686,9 +4689,9 @@
       <c r="D8" s="1">
         <v>0.016</v>
       </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -4779,9 +4782,9 @@
       <c r="D11" s="1">
         <v>0.046</v>
       </c>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -4801,10 +4804,10 @@
       <c r="C12" s="1">
         <v>0.099</v>
       </c>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
@@ -4933,8 +4936,8 @@
       <c r="E16" s="1">
         <v>0.058</v>
       </c>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -4988,9 +4991,9 @@
       <c r="D18" s="1">
         <v>0.024</v>
       </c>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -5019,7 +5022,7 @@
       <c r="F19" s="1">
         <v>0.163</v>
       </c>
-      <c r="G19" s="7"/>
+      <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -5045,8 +5048,8 @@
       <c r="E20" s="1">
         <v>0.161</v>
       </c>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
@@ -5072,8 +5075,8 @@
       <c r="E21" s="1">
         <v>0.028</v>
       </c>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -5129,9 +5132,9 @@
       <c r="D23" s="1">
         <v>0.046</v>
       </c>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
@@ -5157,8 +5160,8 @@
       <c r="E24" s="1">
         <v>3.91</v>
       </c>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
@@ -5187,7 +5190,7 @@
       <c r="F25" s="1">
         <v>0.539</v>
       </c>
-      <c r="G25" s="7"/>
+      <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
@@ -5405,8 +5408,8 @@
       <c r="E32" s="1">
         <v>0.812</v>
       </c>
-      <c r="F32" s="7"/>
-      <c r="G32" s="7"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
@@ -5432,8 +5435,8 @@
       <c r="E33" s="1">
         <v>0.878</v>
       </c>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
@@ -5456,9 +5459,9 @@
       <c r="D34" s="1">
         <v>1.47</v>
       </c>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="7"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
@@ -5484,8 +5487,8 @@
       <c r="E35" s="1">
         <v>2.22</v>
       </c>
-      <c r="F35" s="7"/>
-      <c r="G35" s="7"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
@@ -5495,7 +5498,7 @@
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="19.5">
       <c r="A36" s="1">
         <v>0.514</v>
       </c>
@@ -5514,7 +5517,7 @@
       <c r="F36" s="1">
         <v>0.366</v>
       </c>
-      <c r="G36" s="7"/>
+      <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
@@ -5524,7 +5527,7 @@
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="19.5">
       <c r="A37" s="1">
         <v>0.059</v>
       </c>
@@ -5537,9 +5540,9 @@
       <c r="D37" s="1">
         <v>0.072</v>
       </c>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
@@ -5549,7 +5552,7 @@
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="19.5">
       <c r="A38" s="1">
         <v>0.194</v>
       </c>
@@ -5565,8 +5568,8 @@
       <c r="E38" s="1">
         <v>0.761</v>
       </c>
-      <c r="F38" s="7"/>
-      <c r="G38" s="7"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
@@ -5576,7 +5579,7 @@
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="19.5">
       <c r="A39" s="1">
         <v>0.205</v>
       </c>
@@ -5595,7 +5598,7 @@
       <c r="F39" s="1">
         <v>0.182</v>
       </c>
-      <c r="G39" s="7"/>
+      <c r="G39" s="2"/>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
@@ -5605,7 +5608,7 @@
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="19.5">
       <c r="A40" s="1">
         <v>0.335</v>
       </c>
@@ -5640,7 +5643,7 @@
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="19.5">
       <c r="A41" s="1">
         <v>0.16</v>
       </c>
@@ -5673,7 +5676,7 @@
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="19.5">
       <c r="A42" s="1">
         <v>0.118</v>
       </c>
@@ -5692,7 +5695,7 @@
       <c r="F42" s="1">
         <v>0.144</v>
       </c>
-      <c r="G42" s="7"/>
+      <c r="G42" s="2"/>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
@@ -5702,7 +5705,7 @@
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="19.5">
       <c r="A43" s="1">
         <v>0.621</v>
       </c>
@@ -5721,7 +5724,7 @@
       <c r="F43" s="1">
         <v>0.288</v>
       </c>
-      <c r="G43" s="7"/>
+      <c r="G43" s="2"/>
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
@@ -5731,7 +5734,7 @@
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="19.5">
       <c r="A44" s="1">
         <v>0.466</v>
       </c>
@@ -5747,8 +5750,8 @@
       <c r="E44" s="1">
         <v>0.472</v>
       </c>
-      <c r="F44" s="7"/>
-      <c r="G44" s="7"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
@@ -5758,7 +5761,7 @@
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="19.5">
       <c r="A45" s="1">
         <v>3.35</v>
       </c>
@@ -5799,7 +5802,7 @@
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="19.5">
       <c r="A46" s="1">
         <v>0.125</v>
       </c>
@@ -5836,7 +5839,7 @@
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="19.5">
       <c r="A47" s="1">
         <v>0.045</v>
       </c>
@@ -5869,7 +5872,7 @@
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="19.5">
       <c r="A48" s="1">
         <v>0.022</v>
       </c>
@@ -5902,7 +5905,7 @@
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="19.5">
       <c r="A49" s="1">
         <v>0.54</v>
       </c>
@@ -5918,7 +5921,7 @@
       <c r="E49" s="1">
         <v>0.94</v>
       </c>
-      <c r="F49" s="21">
+      <c r="F49" s="20">
         <v>1</v>
       </c>
       <c r="G49" s="1">
@@ -5943,7 +5946,7 @@
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="19.5">
       <c r="A50" s="1">
         <v>0.267</v>
       </c>
@@ -5974,7 +5977,7 @@
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="19.5">
       <c r="A51" s="1">
         <v>0.798</v>
       </c>
@@ -6005,7 +6008,7 @@
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="19.5">
       <c r="A52" s="1">
         <v>0.046</v>
       </c>
@@ -6042,7 +6045,7 @@
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="19.5">
       <c r="A53" s="1">
         <v>0.873</v>
       </c>
@@ -6061,7 +6064,7 @@
       <c r="F53" s="1">
         <v>0.605</v>
       </c>
-      <c r="G53" s="7"/>
+      <c r="G53" s="2"/>
       <c r="H53" s="2"/>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
@@ -6093,7 +6096,7 @@
       <c r="G54" s="1">
         <v>0.877</v>
       </c>
-      <c r="H54" s="21">
+      <c r="H54" s="20">
         <v>1</v>
       </c>
       <c r="I54" s="1">
@@ -6102,7 +6105,7 @@
       <c r="J54" s="1">
         <v>1.05</v>
       </c>
-      <c r="K54" s="21">
+      <c r="K54" s="20">
         <v>1</v>
       </c>
       <c r="L54" s="2"/>
@@ -6193,7 +6196,7 @@
       <c r="F57" s="1">
         <v>0.112</v>
       </c>
-      <c r="G57" s="7"/>
+      <c r="G57" s="2"/>
       <c r="H57" s="2"/>
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
@@ -6286,7 +6289,7 @@
       <c r="F60" s="1">
         <v>0.153</v>
       </c>
-      <c r="G60" s="7"/>
+      <c r="G60" s="2"/>
       <c r="H60" s="2"/>
       <c r="I60" s="2"/>
       <c r="J60" s="2"/>
@@ -6315,7 +6318,7 @@
       <c r="F61" s="1">
         <v>0.134</v>
       </c>
-      <c r="G61" s="7"/>
+      <c r="G61" s="2"/>
       <c r="H61" s="2"/>
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
@@ -6344,7 +6347,7 @@
       <c r="F62" s="1">
         <v>0.13</v>
       </c>
-      <c r="G62" s="7"/>
+      <c r="G62" s="2"/>
       <c r="H62" s="2"/>
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
@@ -6373,7 +6376,7 @@
       <c r="F63" s="1">
         <v>0.6804</v>
       </c>
-      <c r="G63" s="7"/>
+      <c r="G63" s="2"/>
       <c r="H63" s="2"/>
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
@@ -6623,8 +6626,8 @@
       <c r="E70" s="1">
         <v>0.0273</v>
       </c>
-      <c r="F70" s="7"/>
-      <c r="G70" s="7"/>
+      <c r="F70" s="2"/>
+      <c r="G70" s="2"/>
       <c r="H70" s="2"/>
       <c r="I70" s="2"/>
       <c r="J70" s="2"/>
@@ -6650,8 +6653,8 @@
       <c r="E71" s="1">
         <v>0.238</v>
       </c>
-      <c r="F71" s="7"/>
-      <c r="G71" s="7"/>
+      <c r="F71" s="2"/>
+      <c r="G71" s="2"/>
       <c r="H71" s="2"/>
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
@@ -6708,8 +6711,8 @@
       <c r="E73" s="1">
         <v>0.054</v>
       </c>
-      <c r="F73" s="7"/>
-      <c r="G73" s="7"/>
+      <c r="F73" s="2"/>
+      <c r="G73" s="2"/>
       <c r="H73" s="2"/>
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
@@ -6816,7 +6819,7 @@
       <c r="F76" s="1">
         <v>0.076</v>
       </c>
-      <c r="G76" s="7"/>
+      <c r="G76" s="2"/>
       <c r="H76" s="2"/>
       <c r="I76" s="2"/>
       <c r="J76" s="2"/>
@@ -6839,9 +6842,9 @@
       <c r="D77" s="1">
         <v>0.003</v>
       </c>
-      <c r="E77" s="7"/>
-      <c r="F77" s="7"/>
-      <c r="G77" s="7"/>
+      <c r="E77" s="2"/>
+      <c r="F77" s="2"/>
+      <c r="G77" s="2"/>
       <c r="H77" s="2"/>
       <c r="I77" s="2"/>
       <c r="J77" s="2"/>
@@ -6900,8 +6903,8 @@
       <c r="E79" s="1">
         <v>1.65</v>
       </c>
-      <c r="F79" s="7"/>
-      <c r="G79" s="7"/>
+      <c r="F79" s="2"/>
+      <c r="G79" s="2"/>
       <c r="H79" s="2"/>
       <c r="I79" s="2"/>
       <c r="J79" s="2"/>
@@ -7172,8 +7175,8 @@
       <c r="E87" s="1">
         <v>0.18919999999999998</v>
       </c>
-      <c r="F87" s="7"/>
-      <c r="G87" s="7"/>
+      <c r="F87" s="2"/>
+      <c r="G87" s="2"/>
       <c r="H87" s="2"/>
       <c r="I87" s="2"/>
       <c r="J87" s="2"/>
@@ -7329,8 +7332,8 @@
       <c r="E92" s="1">
         <v>0.182</v>
       </c>
-      <c r="F92" s="7"/>
-      <c r="G92" s="7"/>
+      <c r="F92" s="2"/>
+      <c r="G92" s="2"/>
       <c r="H92" s="2"/>
       <c r="I92" s="2"/>
       <c r="J92" s="2"/>
@@ -7356,8 +7359,8 @@
       <c r="E93" s="1">
         <v>0.418</v>
       </c>
-      <c r="F93" s="7"/>
-      <c r="G93" s="7"/>
+      <c r="F93" s="2"/>
+      <c r="G93" s="2"/>
       <c r="H93" s="2"/>
       <c r="I93" s="2"/>
       <c r="J93" s="2"/>
@@ -7414,8 +7417,8 @@
       <c r="E95" s="1">
         <v>0.1512</v>
       </c>
-      <c r="F95" s="7"/>
-      <c r="G95" s="7"/>
+      <c r="F95" s="2"/>
+      <c r="G95" s="2"/>
       <c r="H95" s="2"/>
       <c r="I95" s="2"/>
       <c r="J95" s="2"/>
@@ -7474,8 +7477,8 @@
       <c r="E97" s="1">
         <v>0.024300000000000002</v>
       </c>
-      <c r="F97" s="7"/>
-      <c r="G97" s="7"/>
+      <c r="F97" s="2"/>
+      <c r="G97" s="2"/>
       <c r="H97" s="2"/>
       <c r="I97" s="2"/>
       <c r="J97" s="2"/>
@@ -7570,17 +7573,17 @@
   <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="27" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="26" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -7611,8 +7614,8 @@
       <c r="I1" s="1">
         <v>142.04999999993015</v>
       </c>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="3"/>
@@ -7640,21 +7643,21 @@
       <c r="I2" s="1">
         <v>0.426</v>
       </c>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="3"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="3" t="s">
@@ -7684,8 +7687,8 @@
       <c r="I4" s="1">
         <v>285.766666666721</v>
       </c>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="3"/>
@@ -7713,21 +7716,21 @@
       <c r="I5" s="1">
         <v>0.139</v>
       </c>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="3"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="3" t="s">
@@ -7772,8 +7775,8 @@
       <c r="C8" s="1">
         <v>1.12</v>
       </c>
-      <c r="D8" s="26">
-        <v>1.3944444444444444</v>
+      <c r="D8" s="25">
+        <v>2.3944444444444444</v>
       </c>
       <c r="E8" s="1">
         <v>1.47</v>
@@ -7810,42 +7813,42 @@
   <dimension ref="A1:AJ100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="27" max="27" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="28" max="28" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="29" max="29" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="30" max="30" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="31" max="31" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="32" max="32" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="33" max="33" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="34" max="34" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="35" max="35" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="36" max="36" style="24" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="33" max="33" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="34" max="34" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="35" max="35" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="36" max="36" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -8018,10 +8021,10 @@
       <c r="C4" s="1">
         <v>130.08</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
@@ -8211,50 +8214,50 @@
       <c r="AJ7" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="8">
+      <c r="A8" s="7">
         <v>54.08</v>
       </c>
-      <c r="B8" s="8">
+      <c r="B8" s="7">
         <v>56.78</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="7">
         <v>65.12</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="7">
         <v>81.75</v>
       </c>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="9"/>
-      <c r="Q8" s="10"/>
-      <c r="R8" s="10"/>
-      <c r="S8" s="10"/>
-      <c r="T8" s="10"/>
-      <c r="U8" s="10"/>
-      <c r="V8" s="10"/>
-      <c r="W8" s="10"/>
-      <c r="X8" s="10"/>
-      <c r="Y8" s="10"/>
-      <c r="Z8" s="10"/>
-      <c r="AA8" s="10"/>
-      <c r="AB8" s="10"/>
-      <c r="AC8" s="10"/>
-      <c r="AD8" s="10"/>
-      <c r="AE8" s="10"/>
-      <c r="AF8" s="10"/>
-      <c r="AG8" s="10"/>
-      <c r="AH8" s="10"/>
-      <c r="AI8" s="10"/>
-      <c r="AJ8" s="10"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="9"/>
+      <c r="R8" s="9"/>
+      <c r="S8" s="9"/>
+      <c r="T8" s="9"/>
+      <c r="U8" s="9"/>
+      <c r="V8" s="9"/>
+      <c r="W8" s="9"/>
+      <c r="X8" s="9"/>
+      <c r="Y8" s="9"/>
+      <c r="Z8" s="9"/>
+      <c r="AA8" s="9"/>
+      <c r="AB8" s="9"/>
+      <c r="AC8" s="9"/>
+      <c r="AD8" s="9"/>
+      <c r="AE8" s="9"/>
+      <c r="AF8" s="9"/>
+      <c r="AG8" s="9"/>
+      <c r="AH8" s="9"/>
+      <c r="AI8" s="9"/>
+      <c r="AJ8" s="9"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1">
@@ -8379,9 +8382,9 @@
       <c r="D11" s="1">
         <v>129.92</v>
       </c>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -8422,10 +8425,10 @@
       <c r="C12" s="1">
         <v>153.53</v>
       </c>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
@@ -8513,56 +8516,56 @@
       <c r="AJ13" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="11">
+      <c r="A14" s="10">
         <v>17.57</v>
       </c>
-      <c r="B14" s="11">
+      <c r="B14" s="10">
         <v>33.7</v>
       </c>
-      <c r="C14" s="11">
+      <c r="C14" s="10">
         <v>58.83</v>
       </c>
-      <c r="D14" s="11">
+      <c r="D14" s="10">
         <v>81.38</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="10">
         <v>105.87</v>
       </c>
-      <c r="F14" s="11">
+      <c r="F14" s="10">
         <v>116.9</v>
       </c>
-      <c r="G14" s="11">
+      <c r="G14" s="10">
         <v>130.12</v>
       </c>
-      <c r="H14" s="12"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="12"/>
-      <c r="M14" s="12"/>
-      <c r="N14" s="12"/>
-      <c r="O14" s="12"/>
-      <c r="P14" s="12"/>
-      <c r="Q14" s="13"/>
-      <c r="R14" s="13"/>
-      <c r="S14" s="13"/>
-      <c r="T14" s="13"/>
-      <c r="U14" s="13"/>
-      <c r="V14" s="13"/>
-      <c r="W14" s="13"/>
-      <c r="X14" s="13"/>
-      <c r="Y14" s="13"/>
-      <c r="Z14" s="13"/>
-      <c r="AA14" s="13"/>
-      <c r="AB14" s="13"/>
-      <c r="AC14" s="13"/>
-      <c r="AD14" s="13"/>
-      <c r="AE14" s="13"/>
-      <c r="AF14" s="13"/>
-      <c r="AG14" s="13"/>
-      <c r="AH14" s="13"/>
-      <c r="AI14" s="13"/>
-      <c r="AJ14" s="13"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="11"/>
+      <c r="O14" s="11"/>
+      <c r="P14" s="11"/>
+      <c r="Q14" s="12"/>
+      <c r="R14" s="12"/>
+      <c r="S14" s="12"/>
+      <c r="T14" s="12"/>
+      <c r="U14" s="12"/>
+      <c r="V14" s="12"/>
+      <c r="W14" s="12"/>
+      <c r="X14" s="12"/>
+      <c r="Y14" s="12"/>
+      <c r="Z14" s="12"/>
+      <c r="AA14" s="12"/>
+      <c r="AB14" s="12"/>
+      <c r="AC14" s="12"/>
+      <c r="AD14" s="12"/>
+      <c r="AE14" s="12"/>
+      <c r="AF14" s="12"/>
+      <c r="AG14" s="12"/>
+      <c r="AH14" s="12"/>
+      <c r="AI14" s="12"/>
+      <c r="AJ14" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="1">
@@ -8623,52 +8626,52 @@
       <c r="AJ15" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="14">
+      <c r="A16" s="13">
         <v>114.22</v>
       </c>
-      <c r="B16" s="14">
+      <c r="B16" s="13">
         <v>129.72</v>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="13">
         <v>129.95</v>
       </c>
-      <c r="D16" s="14">
+      <c r="D16" s="13">
         <v>153.87</v>
       </c>
-      <c r="E16" s="14">
+      <c r="E16" s="13">
         <v>178.28</v>
       </c>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="15"/>
-      <c r="L16" s="15"/>
-      <c r="M16" s="15"/>
-      <c r="N16" s="15"/>
-      <c r="O16" s="15"/>
-      <c r="P16" s="15"/>
-      <c r="Q16" s="16"/>
-      <c r="R16" s="16"/>
-      <c r="S16" s="16"/>
-      <c r="T16" s="16"/>
-      <c r="U16" s="16"/>
-      <c r="V16" s="16"/>
-      <c r="W16" s="16"/>
-      <c r="X16" s="16"/>
-      <c r="Y16" s="16"/>
-      <c r="Z16" s="16"/>
-      <c r="AA16" s="16"/>
-      <c r="AB16" s="16"/>
-      <c r="AC16" s="16"/>
-      <c r="AD16" s="16"/>
-      <c r="AE16" s="16"/>
-      <c r="AF16" s="16"/>
-      <c r="AG16" s="16"/>
-      <c r="AH16" s="16"/>
-      <c r="AI16" s="16"/>
-      <c r="AJ16" s="16"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14"/>
+      <c r="L16" s="14"/>
+      <c r="M16" s="14"/>
+      <c r="N16" s="14"/>
+      <c r="O16" s="14"/>
+      <c r="P16" s="14"/>
+      <c r="Q16" s="15"/>
+      <c r="R16" s="15"/>
+      <c r="S16" s="15"/>
+      <c r="T16" s="15"/>
+      <c r="U16" s="15"/>
+      <c r="V16" s="15"/>
+      <c r="W16" s="15"/>
+      <c r="X16" s="15"/>
+      <c r="Y16" s="15"/>
+      <c r="Z16" s="15"/>
+      <c r="AA16" s="15"/>
+      <c r="AB16" s="15"/>
+      <c r="AC16" s="15"/>
+      <c r="AD16" s="15"/>
+      <c r="AE16" s="15"/>
+      <c r="AF16" s="15"/>
+      <c r="AG16" s="15"/>
+      <c r="AH16" s="15"/>
+      <c r="AI16" s="15"/>
+      <c r="AJ16" s="15"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="1">
@@ -8735,9 +8738,9 @@
       <c r="D18" s="1">
         <v>155.58</v>
       </c>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -8787,7 +8790,7 @@
       <c r="F19" s="1">
         <v>128.43</v>
       </c>
-      <c r="G19" s="7"/>
+      <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -8819,52 +8822,52 @@
       <c r="AJ19" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="17">
+      <c r="A20" s="16">
         <v>18.5</v>
       </c>
-      <c r="B20" s="18">
+      <c r="B20" s="17">
         <v>33</v>
       </c>
-      <c r="C20" s="17">
+      <c r="C20" s="16">
         <v>57.15</v>
       </c>
-      <c r="D20" s="17">
+      <c r="D20" s="16">
         <v>81.5</v>
       </c>
-      <c r="E20" s="17">
+      <c r="E20" s="16">
         <v>106.27</v>
       </c>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="19"/>
-      <c r="J20" s="19"/>
-      <c r="K20" s="19"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="19"/>
-      <c r="N20" s="19"/>
-      <c r="O20" s="19"/>
-      <c r="P20" s="19"/>
-      <c r="Q20" s="20"/>
-      <c r="R20" s="20"/>
-      <c r="S20" s="20"/>
-      <c r="T20" s="20"/>
-      <c r="U20" s="20"/>
-      <c r="V20" s="20"/>
-      <c r="W20" s="20"/>
-      <c r="X20" s="20"/>
-      <c r="Y20" s="20"/>
-      <c r="Z20" s="20"/>
-      <c r="AA20" s="20"/>
-      <c r="AB20" s="20"/>
-      <c r="AC20" s="20"/>
-      <c r="AD20" s="20"/>
-      <c r="AE20" s="20"/>
-      <c r="AF20" s="20"/>
-      <c r="AG20" s="20"/>
-      <c r="AH20" s="20"/>
-      <c r="AI20" s="20"/>
-      <c r="AJ20" s="20"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="18"/>
+      <c r="K20" s="18"/>
+      <c r="L20" s="18"/>
+      <c r="M20" s="18"/>
+      <c r="N20" s="18"/>
+      <c r="O20" s="18"/>
+      <c r="P20" s="18"/>
+      <c r="Q20" s="19"/>
+      <c r="R20" s="19"/>
+      <c r="S20" s="19"/>
+      <c r="T20" s="19"/>
+      <c r="U20" s="19"/>
+      <c r="V20" s="19"/>
+      <c r="W20" s="19"/>
+      <c r="X20" s="19"/>
+      <c r="Y20" s="19"/>
+      <c r="Z20" s="19"/>
+      <c r="AA20" s="19"/>
+      <c r="AB20" s="19"/>
+      <c r="AC20" s="19"/>
+      <c r="AD20" s="19"/>
+      <c r="AE20" s="19"/>
+      <c r="AF20" s="19"/>
+      <c r="AG20" s="19"/>
+      <c r="AH20" s="19"/>
+      <c r="AI20" s="19"/>
+      <c r="AJ20" s="19"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="1">
@@ -8882,8 +8885,8 @@
       <c r="E21" s="1">
         <v>106.47</v>
       </c>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -8981,9 +8984,9 @@
       <c r="D23" s="1">
         <v>154.18</v>
       </c>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
@@ -9030,8 +9033,8 @@
       <c r="E24" s="1">
         <v>106.42</v>
       </c>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
@@ -9081,7 +9084,7 @@
       <c r="F25" s="1">
         <v>106.42</v>
       </c>
-      <c r="G25" s="7"/>
+      <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
@@ -9446,8 +9449,8 @@
       <c r="E32" s="1">
         <v>73.05</v>
       </c>
-      <c r="F32" s="7"/>
-      <c r="G32" s="7"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
@@ -9494,8 +9497,8 @@
       <c r="E33" s="1">
         <v>106.9</v>
       </c>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
@@ -9539,9 +9542,9 @@
       <c r="D34" s="1">
         <v>57.35</v>
       </c>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="7"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
@@ -9588,8 +9591,8 @@
       <c r="E35" s="1">
         <v>105.33</v>
       </c>
-      <c r="F35" s="7"/>
-      <c r="G35" s="7"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
@@ -9639,7 +9642,7 @@
       <c r="F36" s="1">
         <v>67.93333333334886</v>
       </c>
-      <c r="G36" s="7"/>
+      <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
@@ -9683,9 +9686,9 @@
       <c r="D37" s="1">
         <v>92.18333333329065</v>
       </c>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
@@ -9732,8 +9735,8 @@
       <c r="E38" s="1">
         <v>165.81666666670935</v>
       </c>
-      <c r="F38" s="7"/>
-      <c r="G38" s="7"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
@@ -9783,7 +9786,7 @@
       <c r="F39" s="1">
         <v>94.74999999994179</v>
       </c>
-      <c r="G39" s="7"/>
+      <c r="G39" s="2"/>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
@@ -9943,7 +9946,7 @@
       <c r="F42" s="1">
         <v>71.08333333331393</v>
       </c>
-      <c r="G42" s="7"/>
+      <c r="G42" s="2"/>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
@@ -10040,8 +10043,8 @@
       <c r="E44" s="1">
         <v>70.04999999993015</v>
       </c>
-      <c r="F44" s="7"/>
-      <c r="G44" s="7"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
@@ -10601,7 +10604,7 @@
       <c r="F54" s="1">
         <v>151.9000000000815</v>
       </c>
-      <c r="G54" s="7"/>
+      <c r="G54" s="2"/>
       <c r="H54" s="2"/>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
@@ -10817,7 +10820,7 @@
       <c r="F58" s="1">
         <v>115.15000000008149</v>
       </c>
-      <c r="G58" s="7"/>
+      <c r="G58" s="2"/>
       <c r="H58" s="2"/>
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
@@ -10973,7 +10976,7 @@
       <c r="F61" s="1">
         <v>85.483333333279</v>
       </c>
-      <c r="G61" s="7"/>
+      <c r="G61" s="2"/>
       <c r="H61" s="2"/>
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
@@ -11023,7 +11026,7 @@
       <c r="F62" s="1">
         <v>78.96666666667443</v>
       </c>
-      <c r="G62" s="7"/>
+      <c r="G62" s="2"/>
       <c r="H62" s="2"/>
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
@@ -11073,7 +11076,7 @@
       <c r="F63" s="1">
         <v>72.63333333330229</v>
       </c>
-      <c r="G63" s="7"/>
+      <c r="G63" s="2"/>
       <c r="H63" s="2"/>
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
@@ -11123,7 +11126,7 @@
       <c r="F64" s="1">
         <v>73.78333333320916</v>
       </c>
-      <c r="G64" s="7"/>
+      <c r="G64" s="2"/>
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
       <c r="J64" s="2"/>
@@ -11522,8 +11525,8 @@
       <c r="E71" s="1">
         <v>45.766666666720994</v>
       </c>
-      <c r="F71" s="7"/>
-      <c r="G71" s="7"/>
+      <c r="F71" s="2"/>
+      <c r="G71" s="2"/>
       <c r="H71" s="2"/>
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
@@ -11570,8 +11573,8 @@
       <c r="E72" s="1">
         <v>56.850000000034925</v>
       </c>
-      <c r="F72" s="7"/>
-      <c r="G72" s="7"/>
+      <c r="F72" s="2"/>
+      <c r="G72" s="2"/>
       <c r="H72" s="2"/>
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
@@ -11670,8 +11673,8 @@
       <c r="E74" s="1">
         <v>41.43333333340706</v>
       </c>
-      <c r="F74" s="7"/>
-      <c r="G74" s="7"/>
+      <c r="F74" s="2"/>
+      <c r="G74" s="2"/>
       <c r="H74" s="2"/>
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
@@ -11781,7 +11784,7 @@
       <c r="F76" s="1">
         <v>71.33333333343035</v>
       </c>
-      <c r="G76" s="21">
+      <c r="G76" s="20">
         <v>84</v>
       </c>
       <c r="H76" s="1">
@@ -11841,7 +11844,7 @@
       <c r="F77" s="1">
         <v>82.66666666668607</v>
       </c>
-      <c r="G77" s="7"/>
+      <c r="G77" s="2"/>
       <c r="H77" s="2"/>
       <c r="I77" s="2"/>
       <c r="J77" s="2"/>
@@ -11885,9 +11888,9 @@
       <c r="D78" s="1">
         <v>36.18333333340706</v>
       </c>
-      <c r="E78" s="7"/>
-      <c r="F78" s="7"/>
-      <c r="G78" s="7"/>
+      <c r="E78" s="2"/>
+      <c r="F78" s="2"/>
+      <c r="G78" s="2"/>
       <c r="H78" s="2"/>
       <c r="I78" s="2"/>
       <c r="J78" s="2"/>
@@ -11988,8 +11991,8 @@
       <c r="E80" s="1">
         <v>61.28333333332557</v>
       </c>
-      <c r="F80" s="7"/>
-      <c r="G80" s="7"/>
+      <c r="F80" s="2"/>
+      <c r="G80" s="2"/>
       <c r="H80" s="2"/>
       <c r="I80" s="2"/>
       <c r="J80" s="2"/>
@@ -12428,8 +12431,8 @@
       <c r="E88" s="1">
         <v>60.93333333340706</v>
       </c>
-      <c r="F88" s="7"/>
-      <c r="G88" s="7"/>
+      <c r="F88" s="2"/>
+      <c r="G88" s="2"/>
       <c r="H88" s="2"/>
       <c r="I88" s="2"/>
       <c r="J88" s="2"/>
@@ -12690,8 +12693,8 @@
       <c r="E93" s="1">
         <v>58.750000000116415</v>
       </c>
-      <c r="F93" s="7"/>
-      <c r="G93" s="7"/>
+      <c r="F93" s="2"/>
+      <c r="G93" s="2"/>
       <c r="H93" s="2"/>
       <c r="I93" s="2"/>
       <c r="J93" s="2"/>
@@ -12738,8 +12741,8 @@
       <c r="E94" s="1">
         <v>53.60000000009313</v>
       </c>
-      <c r="F94" s="7"/>
-      <c r="G94" s="7"/>
+      <c r="F94" s="2"/>
+      <c r="G94" s="2"/>
       <c r="H94" s="2"/>
       <c r="I94" s="2"/>
       <c r="J94" s="2"/>
@@ -12838,8 +12841,8 @@
       <c r="E96" s="1">
         <v>56.08333333331393</v>
       </c>
-      <c r="F96" s="7"/>
-      <c r="G96" s="7"/>
+      <c r="F96" s="2"/>
+      <c r="G96" s="2"/>
       <c r="H96" s="2"/>
       <c r="I96" s="2"/>
       <c r="J96" s="2"/>
@@ -12940,8 +12943,8 @@
       <c r="E98" s="1">
         <v>61.96666666661622</v>
       </c>
-      <c r="F98" s="7"/>
-      <c r="G98" s="7"/>
+      <c r="F98" s="2"/>
+      <c r="G98" s="2"/>
       <c r="H98" s="2"/>
       <c r="I98" s="2"/>
       <c r="J98" s="2"/>

</xml_diff>